<commit_message>
Calcula frete automaticamente pela malha de rotas (banco_dados)
- roteador.py: motor hub-and-spoke de menor custo que combina trechos
  (CARRETAS 1/2/3) para montar rotas inexistentes diretamente.
- gerar_orcamentos.py: integra o roteamento, preenchendo o custo de cada
  perna e o prazo, mantendo margem/LUCRO, FIPE e coleta/entrega em branco.
- Adiciona banco_dados.xlsx e atualiza os orçamentos gerados.
- 4/6 leads roteados; 2 ficam sem rota (cidade fora da malha).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MFxkgVcDQpZ99TVQnrhozZ
</commit_message>
<xml_diff>
--- a/orcamentos_gerados/Orcamento_ATUS_EUGENIO_ALVES_DA_SILVA.xlsx
+++ b/orcamentos_gerados/Orcamento_ATUS_EUGENIO_ALVES_DA_SILVA.xlsx
@@ -4085,7 +4085,9 @@
           <t>CARRETA 1</t>
         </is>
       </c>
-      <c r="K7" s="314" t="n"/>
+      <c r="K7" s="314" t="n">
+        <v>1500</v>
+      </c>
       <c r="L7" s="20" t="n"/>
       <c r="M7" s="18" t="n"/>
       <c r="N7" s="3" t="n"/>
@@ -4238,7 +4240,9 @@
           <t>CARRETA 2</t>
         </is>
       </c>
-      <c r="K8" s="315" t="n"/>
+      <c r="K8" s="315" t="n">
+        <v>1200</v>
+      </c>
       <c r="L8" s="20" t="n"/>
       <c r="M8" s="21" t="inlineStr">
         <is>
@@ -6693,7 +6697,11 @@
       </c>
       <c r="F23" s="332" t="n"/>
       <c r="G23" s="333" t="n"/>
-      <c r="H23" s="353" t="n"/>
+      <c r="H23" s="353" t="inlineStr">
+        <is>
+          <t>12 dias (confirmar)</t>
+        </is>
+      </c>
       <c r="I23" s="325" t="n"/>
       <c r="K23" s="195" t="n"/>
       <c r="L23" s="303" t="n"/>

</xml_diff>